<commit_message>
fix: move tracker notes out of the append path
The three note lines sat directly under the runs table, so auto-logged
runs would append below them instead of continuing the table. Notes now
live in column Q; the next run appends at row 9.
</commit_message>
<xml_diff>
--- a/training_runs.xlsx
+++ b/training_runs.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -499,6 +499,7 @@
     <col width="10" customWidth="1" min="13" max="13"/>
     <col width="32" customWidth="1" min="14" max="14"/>
     <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="110" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -636,6 +637,11 @@
           <t>First run, full resolution</t>
         </is>
       </c>
+      <c r="Q2" s="5" t="inlineStr">
+        <is>
+          <t>Runs from 2026-08-26 onward exclude the clinical holdout subjects (11192502, PLUCSD004, PLUCSD009) — see holdout_subjects.json.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -693,6 +699,11 @@
       <c r="O3" s="4" t="inlineStr">
         <is>
           <t>3 labels missing (sync issue)</t>
+        </is>
+      </c>
+      <c r="Q3" s="5" t="inlineStr">
+        <is>
+          <t>New rows are appended automatically by scripts/train_seg.py at the end of each run (falls back to training_runs.csv if openpyxl is missing on that machine).</t>
         </is>
       </c>
     </row>
@@ -738,6 +749,11 @@
           <t>Run discarded / not recorded</t>
         </is>
       </c>
+      <c r="Q4" s="5" t="inlineStr">
+        <is>
+          <t>Only the Notes column is meant for hand-editing; all other values come from the training script.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -960,27 +976,6 @@
       <c r="O8" s="2" t="inlineStr">
         <is>
           <t>ACTIVE model. Best PC run</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>Runs from 2026-08-26 onward exclude the clinical holdout subjects (11192502, PLUCSD004, PLUCSD009) — see holdout_subjects.json.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>New rows are appended automatically by scripts/train_seg.py at the end of each run (falls back to training_runs.csv if openpyxl is missing on that machine).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>Only the Notes column is meant for hand-editing; all other values come from the training script.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: one-keystroke correction loop + full retrain-cycle support
The correct-20 / retrain / re-prelabel loop had a silent blocker: Panel 10
never passed --overwrite, so after retraining the old model's stale drafts
were kept. Pre-labeling now always refreshes unverified drafts from the
active model, and a new 'Pre-Label ALL Subjects' button (prelabel.py --all)
regenerates every draft in one click after training.

Correction QoL: 'Save + Next Unreviewed' button and a global Ctrl/Cmd+
Shift+D shortcut save the current corrections, load the next draft, and
open Segment Editor — one keystroke per image. Panel 5 progress line now
also shows global verified/draft counts across all subjects. prelabel.py
prints one line per image so the progress bar actually moves.

scripts/eval_verified.py scores any model against all verified masks per
subject (holdout tagged separately), optional side-by-side overlay PNGs,
and --log appends results to an 'Eval History' sheet in training_runs.xlsx.
</commit_message>
<xml_diff>
--- a/training_runs.xlsx
+++ b/training_runs.xlsx
@@ -1811,7 +1811,7 @@
         <v>5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
@@ -1836,7 +1836,7 @@
         <v>5</v>
       </c>
       <c r="D10" s="2" t="n">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
@@ -1861,7 +1861,7 @@
         <v>5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
@@ -1886,7 +1886,7 @@
         <v>5</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
@@ -1911,7 +1911,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="12" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
@@ -1936,7 +1936,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="12" t="n">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="E14" s="12" t="inlineStr">
         <is>
@@ -2021,10 +2021,11 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Snapshot 2026-08-26. Verified = human-corrected masks in masks/ (training data). Draft = unreviewed model proposals in masks_draft/ (never trained on). Orange rows = clinical holdout, excluded from all training; the 11192502 drafts exist only to be corrected into evaluation ground truth.</t>
+          <t>Snapshot 2026-08-26 (updated: every image now has a draft or verified mask; 1 cine-loop DICOM in 11192502 unprocessable). Verified = human-corrected masks in masks/ (training data). Draft = unreviewed model proposals in masks_draft/ (never trained on). Orange rows = clinical holdout, excluded from all training; the 11192502 drafts exist only to be corrected into evaluation ground truth.</t>
         </is>
       </c>
     </row>

</xml_diff>